<commit_message>
feat: implement Paldea routes & generate regional XLSX files\n\n- Add `paldeaRoutes.js` and `paldeaMapCoordinates.js` to `config/` derived from raw user input.\n- Add Region 10 (Paldea) to `pokedexIndexes.js` (Gen 9 ids 906-1025).\n- Generated regional Excel data files (`.xlsx`) for Regions 6 through 10, populated with validation data, calculated rarity formatting, challenge/unlock associations, and traced base evolution obtainability for unplaced Pokemon.
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/9_Hisui_Data.xlsx
+++ b/9_Hisui_Data.xlsx
@@ -399,20 +399,1256 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:A2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Route</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:E72"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Challenge Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Requisite</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Reward Map</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Reward Challenge</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Reward Gift</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Challenge 3</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Horseshoe Plains</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Challenge 4</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Deertrack Path</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Challenge 5</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Deertrack Heights</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Challenge 6</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Gym - Kleavor, Droning Meadow, Grueling Grove</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Challenge 7</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Earn Kleavor Badge</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Oreburrow Tunnel</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Challenge 8</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Nature’s Pantry</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Challenge 9</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C8" t="str">
+        <v>The Heartwood North</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Challenge 10</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C9" t="str">
+        <v>The Heartwood South</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Challenge 11</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Golden Lowlands North</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Challenge 12</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Golden Lowlands South</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Challenge 13</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Gapejaw Bog North</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Challenge 14</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Gapejaw Bog South</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Challenge 15</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Gym - Lilligant, Obsidian Falls</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Challenge 16</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Earn Lilligant Badge</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Ursa's Ring</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Challenge 17</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Sludge Mound</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Challenge 18</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Scarlet Bog</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Challenge 19</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Bolderoll Slope</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Challenge 20</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Holm of Trials</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Challenge 21</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Crossing Slope</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Challenge 22</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Bathers' Lagoon</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Challenge 23</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Castaway Shore</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Challenge 24</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Deadwood Haunt</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Challenge 25</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Gym - Arcanine</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Challenge 26</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Earn Arcanine Badge</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Veilstone Cape, Gym - Warden Ingo</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Challenge 27</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Tranquility Cove</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Challenge 28</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Islespy Shore</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Challenge 29</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Firespit Island</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Challenge 30</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Spring Path</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Challenge 31</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Celestica Trail</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Challenge 32</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Celestica Ruins</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Challenge 33</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Sacred Plaza</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Challenge 34</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Stonetooth Rows</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Challenge 35</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Primeval Grotto</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Challenge 36</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Gym - Electrode</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Challenge 37</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Earn Electrode Badge</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Clamberclaw Cliffs, Coronet Highlands Fishing Spot</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Challenge 38</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Coronet Highlands</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Challenge 39</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Fabled Spring</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Challenge 40</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Whiteout Valley</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Challenge 41</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Bonechill Wastes North</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Challenge 42</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Bonechill Wastes South</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Challenge 43</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Arena's Approach</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Challenge 44</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Glacier Terrace</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Challenge 45</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Heart's Crag</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Challenge 46</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Snowpoint Temple</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Challenge 47</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Gym - Avalugg</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Extra Challenge A 1</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Earn Warden Ingo Badge</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Obsidian Fieldlands Fishing Spot</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Extra Challenge A 2</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Cobalt Coastlands Fishing Spot</v>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Extra Challenge A 3</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Crimson Mirelands Fishing Spot</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Extra Challenge A 4</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Ginkgo Landing</v>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Extra Challenge A 5</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Shrouded Ruins</v>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Extra Challenge A 6</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Sandgem Flats South</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Extra Challenge A 7</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Ramanas Island South</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Extra Challenge A 8</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Sandgem Flats North</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Extra Challenge B 1</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Cloudpool Ridge North</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Extra Challenge B 2</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Cloudpool Ridge South</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Extra Challenge B 3</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Space-Time Distortion</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Extra Challenge C 1</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Seagrass Haven</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Extra Challenge C 2</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Moonview Arena</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Extra Challenge D 1</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Worn Bridge</v>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Extra Challenge D 2</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Incarnate Fields</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Extra Challenge E 1</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Lake Valor</v>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Extra Challenge E 2</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Lake of Trials</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Extra Challenge F 1</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Defeat 10 in undefined</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Gym of Etertime</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Challenge 48</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Earn Avalugg Badge</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Etertime Storm, Wayward Cave, Alabaster Icelands Fishing Spot, Lake Verity, Etertime Storm</v>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Extra Challenge B 4</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Catch Species: undefined xundefined, undefined xundefined, undefined xundefined, undefined xundefined, undefined xundefined</v>
+      </c>
+      <c r="C66" t="str">
+        <v/>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Extra Challenge C 3</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Catch Species: undefined xundefined, undefined xundefined, undefined xundefined</v>
+      </c>
+      <c r="C67" t="str">
+        <v/>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Extra Challenge D 3</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Catch Species: undefined xundefined, undefined xundefined, undefined xundefined, undefined xundefined</v>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Extra Challenge E 3</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Catch Species: undefined xundefined, undefined xundefined, undefined xundefined</v>
+      </c>
+      <c r="C69" t="str">
+        <v/>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Extra Challenge F 2</v>
+      </c>
+      <c r="B70" t="str">
+        <v>{"defeatMultipleSpecific":[{"name":"Adam"},{"name":"Irida"}]}</v>
+      </c>
+      <c r="C70" t="str">
+        <v/>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Key to Etertime Citadel</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Complete Extra Challenge C 3, Extra Challenge D 3, Extra Challenge E 3, Extra Challenge F 2</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Etertime Citadel</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Etertime Citadel</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Catch Species: undefined xundefined, undefined xundefined, undefined xundefined, undefined xundefined</v>
+      </c>
+      <c r="C72" t="str">
+        <v/>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E72"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>